<commit_message>
auto: timetable update from Sadashiv Bhimanna <sadashiv.bhimanna@nmims.edu>
</commit_message>
<xml_diff>
--- a/downloads/19.10.2026 to25.10.2026.xlsx
+++ b/downloads/19.10.2026 to25.10.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sadashiv.bhimanna\Desktop\2026-27\Trim V\Next week time table trim V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783C390E-A8B5-494E-AFD9-5BFB7C0A7783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F486B046-99D8-44E0-AF88-A31377CB3320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="66">
   <si>
     <t>Day/
 Time</t>
@@ -219,24 +219,12 @@
     <t>5:10 to 6:10 pm</t>
   </si>
   <si>
-    <t>IBDiv A
-Rescheduled class
-Dr Narender Vunyale
-L07, 2nd floor</t>
-  </si>
-  <si>
     <t>CT-B
 Rescheduled class
 Dr Dileep Kumar
 L06,2nd floor</t>
   </si>
   <si>
-    <t>IBDiv B
-Rescheduled class
-Dr Narender Vunyale
-L07, 2nd floor</t>
-  </si>
-  <si>
     <t>MACR 
 (6:00 to 7:30pm)
 L07, 2nd floor
@@ -259,9 +247,6 @@
   </si>
   <si>
     <t>Placement activity</t>
-  </si>
-  <si>
-    <t>Placement Activity</t>
   </si>
   <si>
     <t>6:00 to 7:30 pm</t>
@@ -298,6 +283,27 @@
 (6:00pm to 7:30 pm)
 L06, 2nd floor
 Prof Murtuza</t>
+  </si>
+  <si>
+    <t>IB Div-A
+Rescheduled class
+Dr Narender Vunyale
+L07, 2nd floor</t>
+  </si>
+  <si>
+    <t>IB Div-B
+Rescheduled class
+Dr Narender Vunyale
+L07, 2nd floor</t>
+  </si>
+  <si>
+    <t>SM 
+(7:35pm to 9:05 pm)
+L06, 2nd floor
+Prof Murtuza</t>
+  </si>
+  <si>
+    <t>7:35 to 9:05 pm</t>
   </si>
 </sst>
 </file>
@@ -436,7 +442,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="45">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -639,19 +645,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -985,6 +978,47 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -994,7 +1028,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1018,7 +1052,7 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="3" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1027,99 +1061,86 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -1127,33 +1148,64 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1167,7 +1219,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1179,7 +1231,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1188,32 +1240,20 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1500,7 +1540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
@@ -1511,24 +1551,24 @@
     <col min="8" max="8" width="19.7109375" customWidth="1"/>
     <col min="9" max="9" width="17.7109375" customWidth="1"/>
     <col min="10" max="10" width="22.140625" customWidth="1"/>
-    <col min="11" max="11" width="19" customWidth="1"/>
+    <col min="11" max="11" width="23.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
+    <row r="1" spans="1:11" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="74" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-    </row>
-    <row r="2" spans="1:10" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+    </row>
+    <row r="2" spans="1:11" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1550,16 +1590,19 @@
       <c r="G2" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="72" t="s">
+      <c r="H2" s="84" t="s">
         <v>49</v>
       </c>
-      <c r="I2" s="73"/>
-      <c r="J2" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="64" t="s">
+      <c r="I2" s="85"/>
+      <c r="J2" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="K2" s="68" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="76" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="6"/>
@@ -1569,23 +1612,24 @@
       <c r="D3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="65" t="s">
+      <c r="E3" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="57" t="s">
+      <c r="G3" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="I3" s="61"/>
-      <c r="J3" s="44"/>
-    </row>
-    <row r="4" spans="1:10" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="64"/>
+      <c r="H3" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="55"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="69"/>
+    </row>
+    <row r="4" spans="1:11" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="76"/>
       <c r="B4" s="7"/>
       <c r="C4" s="14" t="s">
         <v>9</v>
@@ -1593,179 +1637,187 @@
       <c r="D4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="66"/>
+      <c r="E4" s="78"/>
       <c r="F4" s="8"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="39"/>
-    </row>
-    <row r="5" spans="1:10" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="64" t="s">
+      <c r="G4" s="52"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="70"/>
+    </row>
+    <row r="5" spans="1:11" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="76" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="6"/>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="86" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="87"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="86" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" s="87"/>
+      <c r="H5" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="I5" s="54" t="s">
+        <v>59</v>
+      </c>
+      <c r="J5" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="75"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="74" t="s">
-        <v>57</v>
-      </c>
-      <c r="G5" s="75"/>
-      <c r="H5" s="59" t="s">
+      <c r="K5" s="70"/>
+    </row>
+    <row r="6" spans="1:11" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="76"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="88"/>
+      <c r="D6" s="89"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="89"/>
+      <c r="H6" s="47" t="s">
+        <v>60</v>
+      </c>
+      <c r="I6" s="48"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="70"/>
+    </row>
+    <row r="7" spans="1:11" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="76" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="80"/>
+      <c r="F7" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="50"/>
+      <c r="J7" s="63"/>
+      <c r="K7" s="70"/>
+    </row>
+    <row r="8" spans="1:11" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="76"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="80"/>
+      <c r="F8" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="23"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="70"/>
+    </row>
+    <row r="9" spans="1:11" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="82" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="56"/>
+      <c r="C9" s="60" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="81"/>
+      <c r="F9" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="57"/>
+      <c r="I9" s="49"/>
+      <c r="K9" s="70"/>
+    </row>
+    <row r="10" spans="1:11" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="83"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="81"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="58"/>
+      <c r="I10" s="36"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="71"/>
+    </row>
+    <row r="11" spans="1:11" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="43" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="44"/>
+      <c r="C11" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="32"/>
+      <c r="F11" s="34" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="H11" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" s="38"/>
+      <c r="J11" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="I5" s="60" t="s">
-        <v>62</v>
-      </c>
-      <c r="J5" s="42" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="64"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="76"/>
-      <c r="D6" s="77"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="77"/>
-      <c r="H6" s="52" t="s">
-        <v>63</v>
-      </c>
-      <c r="I6" s="53"/>
-      <c r="J6" s="39"/>
-    </row>
-    <row r="7" spans="1:10" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="64" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="68"/>
-      <c r="F7" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="44"/>
-    </row>
-    <row r="8" spans="1:10" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="64"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="39"/>
-    </row>
-    <row r="9" spans="1:10" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="70" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="78" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="79"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" s="54"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="20" t="s">
+      <c r="K11" s="73" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="69" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="45" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="71"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="80"/>
-      <c r="D10" s="81"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="40" t="s">
-        <v>51</v>
-      </c>
-      <c r="G10" s="39"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="8"/>
-    </row>
-    <row r="11" spans="1:10" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="49"/>
-      <c r="C11" s="33" t="s">
+      <c r="B12" s="46"/>
+      <c r="C12" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D12" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="35"/>
-      <c r="F11" s="37" t="s">
+      <c r="E12" s="32"/>
+      <c r="F12" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="G11" s="38" t="s">
+      <c r="G12" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="33" t="s">
+      <c r="H12" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="41"/>
-      <c r="J11" s="34" t="s">
+      <c r="I12" s="38"/>
+      <c r="J12" s="67" t="s">
+        <v>61</v>
+      </c>
+      <c r="K12" s="72" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="69" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="50" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="51"/>
-      <c r="C12" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="35"/>
-      <c r="F12" s="37" t="s">
-        <v>44</v>
-      </c>
-      <c r="G12" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="H12" s="33" t="s">
-        <v>48</v>
-      </c>
-      <c r="I12" s="41"/>
-      <c r="J12" s="34" t="s">
-        <v>64</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="E3:E10"/>
@@ -1775,7 +1827,6 @@
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="F5:G6"/>
-    <mergeCell ref="C9:D10"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>